<commit_message>
Standardize DBMS Unit 3 lessons and update MCQ banks
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Unit 2 - Data Types and Operators/Unit 2 - Data Types and Operators - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Unit 2 - Data Types and Operators/Unit 2 - Data Types and Operators - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - Unit 2" sheetId="1" r:id="Rc74a7e48418c4da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - Unit 2" sheetId="1" r:id="R2a8de5d9644840bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,12 +26,27 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -45,7 +60,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -57,6 +72,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -394,55 +418,55 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="8" t="str">
         <x:v>title</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="8" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="8" t="str">
         <x:v>explanation</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="8" t="str">
         <x:v>score</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="8" t="str">
         <x:v>status</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" s="8" t="str">
         <x:v>difficulty</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="str">
+      <x:c r="G1" s="8" t="str">
         <x:v>bloomTaxonomy</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="str">
+      <x:c r="H1" s="8" t="str">
         <x:v>tags</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="str">
+      <x:c r="I1" s="8" t="str">
         <x:v>subjects</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="str">
+      <x:c r="J1" s="8" t="str">
         <x:v>topics</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="str">
+      <x:c r="K1" s="8" t="str">
         <x:v>subTopics</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="str">
+      <x:c r="L1" s="8" t="str">
         <x:v>companies</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="str">
+      <x:c r="M1" s="8" t="str">
         <x:v>option1</x:v>
       </x:c>
-      <x:c r="N1" s="3" t="str">
+      <x:c r="N1" s="8" t="str">
         <x:v>option2</x:v>
       </x:c>
-      <x:c r="O1" s="3" t="str">
+      <x:c r="O1" s="8" t="str">
         <x:v>option3</x:v>
       </x:c>
-      <x:c r="P1" s="3" t="str">
+      <x:c r="P1" s="8" t="str">
         <x:v>option4</x:v>
       </x:c>
-      <x:c r="Q1" s="3" t="str">
+      <x:c r="Q1" s="8" t="str">
         <x:v>answer</x:v>
       </x:c>
     </x:row>
@@ -468,7 +492,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F2" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G2" s="4" t="str">
         <x:v>analyze</x:v>
@@ -738,7 +762,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
         <x:v>apply</x:v>
@@ -848,7 +872,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G9" s="4" t="str">
         <x:v>apply</x:v>
@@ -1017,7 +1041,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G12" s="4" t="str">
         <x:v>apply</x:v>
@@ -1072,7 +1096,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F13" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G13" s="4" t="str">
         <x:v>analyze</x:v>
@@ -1444,7 +1468,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F20" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G20" s="4" t="str">
         <x:v>apply</x:v>
@@ -1715,7 +1739,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F25" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G25" s="4" t="str">
         <x:v>analyze</x:v>
@@ -1770,7 +1794,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F26" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G26" s="4" t="str">
         <x:v>evaluate</x:v>
@@ -1821,7 +1845,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G27" s="4" t="str">
         <x:v>analyze</x:v>
@@ -1876,7 +1900,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G28" s="4" t="str">
         <x:v>apply</x:v>
@@ -1928,7 +1952,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F29" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G29" s="4" t="str">
         <x:v>apply</x:v>
@@ -2036,7 +2060,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F31" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G31" s="4" t="str">
         <x:v>analyze</x:v>
@@ -2088,7 +2112,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F32" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G32" s="4" t="str">
         <x:v>apply</x:v>
@@ -2139,7 +2163,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F33" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G33" s="4" t="str">
         <x:v>apply</x:v>
@@ -2245,7 +2269,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F35" s="4" t="str">
-        <x:v>easy</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G35" s="4" t="str">
         <x:v>analyze</x:v>
@@ -2408,7 +2432,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F38" s="4" t="str">
-        <x:v>hard</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="G38" s="4" t="str">
         <x:v>apply</x:v>
@@ -2459,7 +2483,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F39" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>easy</x:v>
       </x:c>
       <x:c r="G39" s="4" t="str">
         <x:v>apply</x:v>
@@ -2570,7 +2594,7 @@
         <x:v>published</x:v>
       </x:c>
       <x:c r="F41" s="4" t="str">
-        <x:v>medium</x:v>
+        <x:v>hard</x:v>
       </x:c>
       <x:c r="G41" s="4" t="str">
         <x:v>evaluate</x:v>
@@ -2607,7 +2631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24d9e88b1df84151"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64a92508301e4132"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>